<commit_message>
data: 2026-10-14 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3516,6 +3516,37 @@
         <v>96.62</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="n">
+        <v>9131</v>
+      </c>
+      <c r="C100" s="3" t="n">
+        <v>10097707.36</v>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>9087132.880000001</v>
+      </c>
+      <c r="E100" s="3" t="n">
+        <v>1010574.48</v>
+      </c>
+      <c r="F100" s="4" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="G100" s="4" t="n">
+        <v>1105.87</v>
+      </c>
+      <c r="H100" s="5" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="I100" s="5" t="n">
+        <v>96.66</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-15 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3547,6 +3547,37 @@
         <v>96.66</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="n">
+        <v>9127</v>
+      </c>
+      <c r="C101" s="3" t="n">
+        <v>10072568.08</v>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>9070742.789999999</v>
+      </c>
+      <c r="E101" s="3" t="n">
+        <v>1001825.29</v>
+      </c>
+      <c r="F101" s="4" t="n">
+        <v>3.8075</v>
+      </c>
+      <c r="G101" s="4" t="n">
+        <v>1103.6</v>
+      </c>
+      <c r="H101" s="5" t="n">
+        <v>87.45999999999999</v>
+      </c>
+      <c r="I101" s="5" t="n">
+        <v>96.67</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>